<commit_message>
Updated code quality rules and rel rating
</commit_message>
<xml_diff>
--- a/help/implementing/cloud-manager/assets/CodeQuality-rules-latest-CS.xlsx
+++ b/help/implementing/cloud-manager/assets/CodeQuality-rules-latest-CS.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10711"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10111"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://adobe-my.sharepoint.com/personal/jedelson_adobe_com/Documents/AMS/Pathlight/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="44" documentId="13_ncr:1_{66F76743-C75B-7A4F-8D1D-1800026AF33A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{48FCA269-EBEE-424E-9FAF-C6A74825CA71}"/>
+  <xr:revisionPtr revIDLastSave="49" documentId="13_ncr:1_{66F76743-C75B-7A4F-8D1D-1800026AF33A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C70E7FB7-2C1A-8D4E-B017-C7832267726A}"/>
   <bookViews>
     <workbookView xWindow="-38400" yWindow="-1360" windowWidth="38400" windowHeight="14680" xr2:uid="{38B21097-AA8D-8C49-8C0F-A8DA08168C4C}"/>
   </bookViews>
@@ -858,9 +858,6 @@
     <t>Product interfaces annotated with @ProviderType should not be implemented by custom code.</t>
   </si>
   <si>
-    <t>BannedPaths</t>
-  </si>
-  <si>
     <t>Customer packages should not install content under /libs</t>
   </si>
   <si>
@@ -1015,6 +1012,9 @@
   </si>
   <si>
     <t>Custom Lucene Oak Indexes must not be synchronous</t>
+  </si>
+  <si>
+    <t>BannedPath</t>
   </si>
 </sst>
 </file>
@@ -1984,10 +1984,10 @@
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>277</v>
+        <v>299</v>
       </c>
       <c r="B35" t="s">
-        <v>278</v>
+        <v>300</v>
       </c>
       <c r="C35" t="s">
         <v>179</v>
@@ -1995,13 +1995,16 @@
       <c r="D35" t="s">
         <v>153</v>
       </c>
+      <c r="E35" t="s">
+        <v>290</v>
+      </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>300</v>
+        <v>317</v>
       </c>
       <c r="B36" t="s">
-        <v>301</v>
+        <v>318</v>
       </c>
       <c r="C36" t="s">
         <v>179</v>
@@ -2010,15 +2013,15 @@
         <v>153</v>
       </c>
       <c r="E36" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>318</v>
+        <v>325</v>
       </c>
       <c r="B37" t="s">
-        <v>319</v>
+        <v>328</v>
       </c>
       <c r="C37" t="s">
         <v>179</v>
@@ -2027,7 +2030,7 @@
         <v>153</v>
       </c>
       <c r="E37" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.2">
@@ -2035,7 +2038,7 @@
         <v>326</v>
       </c>
       <c r="B38" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="C38" t="s">
         <v>179</v>
@@ -2044,15 +2047,15 @@
         <v>153</v>
       </c>
       <c r="E38" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>327</v>
+        <v>323</v>
       </c>
       <c r="B39" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="C39" t="s">
         <v>179</v>
@@ -2061,24 +2064,21 @@
         <v>153</v>
       </c>
       <c r="E39" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>324</v>
+        <v>329</v>
       </c>
       <c r="B40" t="s">
-        <v>325</v>
+        <v>277</v>
       </c>
       <c r="C40" t="s">
         <v>179</v>
       </c>
       <c r="D40" t="s">
-        <v>153</v>
-      </c>
-      <c r="E40" t="s">
-        <v>291</v>
+        <v>159</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.2">
@@ -2587,10 +2587,10 @@
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
+        <v>278</v>
+      </c>
+      <c r="B71" t="s">
         <v>279</v>
-      </c>
-      <c r="B71" t="s">
-        <v>280</v>
       </c>
       <c r="C71" t="s">
         <v>179</v>
@@ -2601,10 +2601,10 @@
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
+        <v>280</v>
+      </c>
+      <c r="B72" t="s">
         <v>281</v>
-      </c>
-      <c r="B72" t="s">
-        <v>282</v>
       </c>
       <c r="C72" t="s">
         <v>179</v>
@@ -2615,10 +2615,10 @@
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
+        <v>282</v>
+      </c>
+      <c r="B73" t="s">
         <v>283</v>
-      </c>
-      <c r="B73" t="s">
-        <v>284</v>
       </c>
       <c r="C73" t="s">
         <v>179</v>
@@ -2629,10 +2629,10 @@
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A74" s="3" t="s">
+        <v>297</v>
+      </c>
+      <c r="B74" s="3" t="s">
         <v>298</v>
-      </c>
-      <c r="B74" s="3" t="s">
-        <v>299</v>
       </c>
       <c r="C74" s="3" t="s">
         <v>179</v>
@@ -3345,10 +3345,10 @@
     </row>
     <row r="116" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A116" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="B116" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C116" t="s">
         <v>226</v>
@@ -3357,15 +3357,15 @@
         <v>175</v>
       </c>
       <c r="E116" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="117" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A117" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="B117" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="C117" t="s">
         <v>226</v>
@@ -3374,15 +3374,15 @@
         <v>175</v>
       </c>
       <c r="E117" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="118" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A118" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B118" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="C118" t="s">
         <v>226</v>
@@ -3391,15 +3391,15 @@
         <v>175</v>
       </c>
       <c r="E118" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="119" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A119" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="B119" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="C119" t="s">
         <v>226</v>
@@ -3408,15 +3408,15 @@
         <v>175</v>
       </c>
       <c r="E119" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="120" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A120" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="B120" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="C120" t="s">
         <v>226</v>
@@ -3425,33 +3425,33 @@
         <v>175</v>
       </c>
       <c r="E120" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="121" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A121" t="s">
+        <v>289</v>
+      </c>
+      <c r="B121" t="s">
+        <v>291</v>
+      </c>
+      <c r="C121" t="s">
+        <v>226</v>
+      </c>
+      <c r="D121" t="s">
+        <v>175</v>
+      </c>
+      <c r="E121" t="s">
         <v>290</v>
-      </c>
-      <c r="B121" t="s">
-        <v>292</v>
-      </c>
-      <c r="C121" t="s">
-        <v>226</v>
-      </c>
-      <c r="D121" t="s">
-        <v>175</v>
-      </c>
-      <c r="E121" t="s">
-        <v>291</v>
       </c>
     </row>
     <row r="122" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A122" t="s">
+        <v>299</v>
+      </c>
+      <c r="B122" t="s">
         <v>300</v>
       </c>
-      <c r="B122" t="s">
-        <v>301</v>
-      </c>
       <c r="C122" t="s">
         <v>226</v>
       </c>
@@ -3459,16 +3459,16 @@
         <v>175</v>
       </c>
       <c r="E122" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="123" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A123" t="s">
+        <v>301</v>
+      </c>
+      <c r="B123" t="s">
         <v>302</v>
       </c>
-      <c r="B123" t="s">
-        <v>303</v>
-      </c>
       <c r="C123" t="s">
         <v>226</v>
       </c>
@@ -3476,16 +3476,16 @@
         <v>175</v>
       </c>
       <c r="E123" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="124" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A124" t="s">
+        <v>303</v>
+      </c>
+      <c r="B124" t="s">
         <v>304</v>
       </c>
-      <c r="B124" t="s">
-        <v>305</v>
-      </c>
       <c r="C124" t="s">
         <v>226</v>
       </c>
@@ -3493,16 +3493,16 @@
         <v>175</v>
       </c>
       <c r="E124" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="125" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A125" t="s">
+        <v>305</v>
+      </c>
+      <c r="B125" t="s">
         <v>306</v>
       </c>
-      <c r="B125" t="s">
-        <v>307</v>
-      </c>
       <c r="C125" t="s">
         <v>226</v>
       </c>
@@ -3510,16 +3510,16 @@
         <v>175</v>
       </c>
       <c r="E125" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="126" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A126" t="s">
+        <v>307</v>
+      </c>
+      <c r="B126" t="s">
         <v>308</v>
       </c>
-      <c r="B126" t="s">
-        <v>309</v>
-      </c>
       <c r="C126" t="s">
         <v>226</v>
       </c>
@@ -3527,16 +3527,16 @@
         <v>175</v>
       </c>
       <c r="E126" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="127" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A127" t="s">
+        <v>309</v>
+      </c>
+      <c r="B127" t="s">
         <v>310</v>
       </c>
-      <c r="B127" t="s">
-        <v>311</v>
-      </c>
       <c r="C127" t="s">
         <v>226</v>
       </c>
@@ -3544,16 +3544,16 @@
         <v>175</v>
       </c>
       <c r="E127" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="128" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A128" t="s">
+        <v>311</v>
+      </c>
+      <c r="B128" t="s">
         <v>312</v>
       </c>
-      <c r="B128" t="s">
-        <v>313</v>
-      </c>
       <c r="C128" t="s">
         <v>226</v>
       </c>
@@ -3561,16 +3561,16 @@
         <v>175</v>
       </c>
       <c r="E128" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="129" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A129" t="s">
+        <v>313</v>
+      </c>
+      <c r="B129" t="s">
         <v>314</v>
       </c>
-      <c r="B129" t="s">
-        <v>315</v>
-      </c>
       <c r="C129" t="s">
         <v>226</v>
       </c>
@@ -3578,16 +3578,16 @@
         <v>175</v>
       </c>
       <c r="E129" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="130" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A130" t="s">
+        <v>315</v>
+      </c>
+      <c r="B130" t="s">
         <v>316</v>
       </c>
-      <c r="B130" t="s">
-        <v>317</v>
-      </c>
       <c r="C130" t="s">
         <v>226</v>
       </c>
@@ -3595,16 +3595,16 @@
         <v>175</v>
       </c>
       <c r="E130" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="131" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A131" t="s">
+        <v>319</v>
+      </c>
+      <c r="B131" t="s">
         <v>320</v>
       </c>
-      <c r="B131" t="s">
-        <v>321</v>
-      </c>
       <c r="C131" t="s">
         <v>226</v>
       </c>
@@ -3612,16 +3612,16 @@
         <v>175</v>
       </c>
       <c r="E131" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="132" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A132" t="s">
+        <v>321</v>
+      </c>
+      <c r="B132" t="s">
         <v>322</v>
       </c>
-      <c r="B132" t="s">
-        <v>323</v>
-      </c>
       <c r="C132" t="s">
         <v>226</v>
       </c>
@@ -3629,7 +3629,7 @@
         <v>175</v>
       </c>
       <c r="E132" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="133" spans="1:5" x14ac:dyDescent="0.2">

</xml_diff>